<commit_message>
Add Market (metro) column to the portfolio data tape (PDF + Excel)
Each asset now shows its market — Houston, TX / Miami, FL (Golden Glades'
"Miami, TX" model typo overridden to FL) — in the asset-level data tape on
both the PDF portfolio page and the Excel dashboard. Shortened the portfolio
total-row market cell so the Asset column keeps its width (no more truncation
of "Pearl Washington").

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0124FZLJoPnoM29DgdDCtmep
</commit_message>
<xml_diff>
--- a/output/Morgan_Recap_Data_Tape.xlsx
+++ b/output/Morgan_Recap_Data_Tape.xlsx
@@ -959,75 +959,80 @@
       </c>
       <c r="D16" s="18" t="inlineStr">
         <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="F16" s="18" t="inlineStr">
         <is>
           <t>Built</t>
         </is>
       </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="G16" s="18" t="inlineStr">
         <is>
           <t>Ask</t>
         </is>
       </c>
-      <c r="G16" s="18" t="inlineStr">
+      <c r="H16" s="18" t="inlineStr">
         <is>
           <t>$/Unit</t>
         </is>
       </c>
-      <c r="H16" s="18" t="inlineStr">
+      <c r="I16" s="18" t="inlineStr">
         <is>
           <t>Occ</t>
         </is>
       </c>
-      <c r="I16" s="18" t="inlineStr">
+      <c r="J16" s="18" t="inlineStr">
         <is>
           <t>Contract /mo</t>
         </is>
       </c>
-      <c r="J16" s="18" t="inlineStr">
+      <c r="K16" s="18" t="inlineStr">
         <is>
           <t>New T/O</t>
         </is>
       </c>
-      <c r="K16" s="18" t="inlineStr">
+      <c r="L16" s="18" t="inlineStr">
         <is>
           <t>T12 NOI</t>
         </is>
       </c>
-      <c r="L16" s="18" t="inlineStr">
+      <c r="M16" s="18" t="inlineStr">
         <is>
           <t>Act Cap</t>
         </is>
       </c>
-      <c r="M16" s="18" t="inlineStr">
+      <c r="N16" s="18" t="inlineStr">
         <is>
           <t>JLL UW Cap</t>
         </is>
       </c>
-      <c r="N16" s="18" t="inlineStr">
+      <c r="O16" s="18" t="inlineStr">
         <is>
           <t>Yr-1 Cap</t>
         </is>
       </c>
-      <c r="O16" s="18" t="inlineStr">
+      <c r="P16" s="18" t="inlineStr">
         <is>
           <t>Exit Cap</t>
         </is>
       </c>
-      <c r="P16" s="18" t="inlineStr">
+      <c r="Q16" s="18" t="inlineStr">
         <is>
           <t>JLL UW LIRR</t>
         </is>
       </c>
-      <c r="Q16" s="18" t="inlineStr">
+      <c r="R16" s="18" t="inlineStr">
         <is>
           <t>EM</t>
         </is>
       </c>
-      <c r="R16" s="17" t="inlineStr">
+      <c r="S16" s="17" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
@@ -1041,46 +1046,51 @@
       </c>
       <c r="B17" s="20" t="n"/>
       <c r="C17" s="20" t="n"/>
-      <c r="D17" s="21" t="n">
+      <c r="D17" s="21" t="inlineStr">
+        <is>
+          <t>Houston, TX</t>
+        </is>
+      </c>
+      <c r="E17" s="21" t="n">
         <v>459</v>
       </c>
-      <c r="E17" s="22" t="n">
+      <c r="F17" s="22" t="n">
         <v>2015</v>
       </c>
-      <c r="F17" s="23" t="n">
+      <c r="G17" s="23" t="n">
         <v>127000000</v>
       </c>
-      <c r="G17" s="24" t="n">
+      <c r="H17" s="24" t="n">
         <v>276688.4531590414</v>
       </c>
-      <c r="H17" s="25" t="n">
+      <c r="I17" s="25" t="n">
         <v>0.9694989106753813</v>
       </c>
-      <c r="I17" s="24" t="n">
+      <c r="J17" s="24" t="n">
         <v>2330.481481481481</v>
       </c>
-      <c r="J17" s="25" t="n">
+      <c r="K17" s="25" t="n">
         <v>0.03463420147578833</v>
       </c>
-      <c r="K17" s="23" t="n">
+      <c r="L17" s="23" t="n">
         <v>6556237</v>
       </c>
-      <c r="L17" s="26" t="n">
+      <c r="M17" s="26" t="n">
         <v>0.05162391338582677</v>
       </c>
-      <c r="M17" s="26" t="n">
+      <c r="N17" s="26" t="n">
         <v>0.05070069856746456</v>
       </c>
-      <c r="N17" s="26" t="n">
+      <c r="O17" s="26" t="n">
         <v>0.05335014871664925</v>
       </c>
-      <c r="O17" s="26" t="n">
+      <c r="P17" s="26" t="n">
         <v>0.05</v>
       </c>
-      <c r="P17" s="25" t="n">
+      <c r="Q17" s="25" t="n">
         <v>0.1629796862069719</v>
       </c>
-      <c r="Q17" s="27" t="n">
+      <c r="R17" s="27" t="n">
         <v>1.999137963456238</v>
       </c>
     </row>
@@ -1092,46 +1102,51 @@
       </c>
       <c r="B18" s="29" t="n"/>
       <c r="C18" s="29" t="n"/>
-      <c r="D18" s="30" t="n">
+      <c r="D18" s="30" t="inlineStr">
+        <is>
+          <t>Miami, FL</t>
+        </is>
+      </c>
+      <c r="E18" s="30" t="n">
         <v>236</v>
       </c>
-      <c r="E18" s="31" t="n">
+      <c r="F18" s="31" t="n">
         <v>2024</v>
       </c>
-      <c r="F18" s="32" t="n">
+      <c r="G18" s="32" t="n">
         <v>85000000</v>
       </c>
-      <c r="G18" s="33" t="n">
+      <c r="H18" s="33" t="n">
         <v>360169.4915254237</v>
       </c>
-      <c r="H18" s="34" t="n">
+      <c r="I18" s="34" t="n">
         <v>0.923728813559322</v>
       </c>
-      <c r="I18" s="33" t="n">
+      <c r="J18" s="33" t="n">
         <v>2528.881355932203</v>
       </c>
-      <c r="J18" s="34" t="n">
+      <c r="K18" s="34" t="n">
         <v>-0.115485050906139</v>
       </c>
-      <c r="K18" s="32" t="n">
+      <c r="L18" s="32" t="n">
         <v>3802396</v>
       </c>
-      <c r="L18" s="35" t="n">
+      <c r="M18" s="35" t="n">
         <v>0.04473407058823529</v>
       </c>
-      <c r="M18" s="35" t="n">
+      <c r="N18" s="35" t="n">
         <v>0.04666074939670589</v>
       </c>
-      <c r="N18" s="35" t="n">
+      <c r="O18" s="35" t="n">
         <v>0.0479255411819897</v>
       </c>
-      <c r="O18" s="35" t="n">
+      <c r="P18" s="35" t="n">
         <v>0.0475</v>
       </c>
-      <c r="P18" s="34" t="n">
+      <c r="Q18" s="34" t="n">
         <v>0.1515156658203647</v>
       </c>
-      <c r="Q18" s="36" t="n">
+      <c r="R18" s="36" t="n">
         <v>1.922478917528772</v>
       </c>
     </row>
@@ -1143,46 +1158,51 @@
       </c>
       <c r="B19" s="20" t="n"/>
       <c r="C19" s="20" t="n"/>
-      <c r="D19" s="21" t="n">
+      <c r="D19" s="21" t="inlineStr">
+        <is>
+          <t>Houston, TX</t>
+        </is>
+      </c>
+      <c r="E19" s="21" t="n">
         <v>322</v>
       </c>
-      <c r="E19" s="22" t="n">
+      <c r="F19" s="22" t="n">
         <v>2016</v>
       </c>
-      <c r="F19" s="23" t="n">
+      <c r="G19" s="23" t="n">
         <v>60000000</v>
       </c>
-      <c r="G19" s="24" t="n">
+      <c r="H19" s="24" t="n">
         <v>186335.4037267081</v>
       </c>
-      <c r="H19" s="25" t="n">
+      <c r="I19" s="25" t="n">
         <v>0.937888198757764</v>
       </c>
-      <c r="I19" s="24" t="n">
+      <c r="J19" s="24" t="n">
         <v>1687.074534161491</v>
       </c>
-      <c r="J19" s="25" t="n">
+      <c r="K19" s="25" t="n">
         <v>-0.1521936575618804</v>
       </c>
-      <c r="K19" s="23" t="n">
+      <c r="L19" s="23" t="n">
         <v>2772820</v>
       </c>
-      <c r="L19" s="26" t="n">
+      <c r="M19" s="26" t="n">
         <v>0.04621366666666667</v>
       </c>
-      <c r="M19" s="26" t="n">
+      <c r="N19" s="26" t="n">
         <v>0.051301136661004</v>
       </c>
-      <c r="N19" s="26" t="n">
+      <c r="O19" s="26" t="n">
         <v>0.05396175469133623</v>
       </c>
-      <c r="O19" s="26" t="n">
+      <c r="P19" s="26" t="n">
         <v>0.05</v>
       </c>
-      <c r="P19" s="25" t="n">
+      <c r="Q19" s="25" t="n">
         <v>0.1766852207761906</v>
       </c>
-      <c r="Q19" s="27" t="n">
+      <c r="R19" s="27" t="n">
         <v>2.144502169992451</v>
       </c>
     </row>
@@ -1194,46 +1214,51 @@
       </c>
       <c r="B20" s="29" t="n"/>
       <c r="C20" s="29" t="n"/>
-      <c r="D20" s="30" t="n">
+      <c r="D20" s="30" t="inlineStr">
+        <is>
+          <t>Houston, TX</t>
+        </is>
+      </c>
+      <c r="E20" s="30" t="n">
         <v>215</v>
       </c>
-      <c r="E20" s="31" t="n">
+      <c r="F20" s="31" t="n">
         <v>2015</v>
       </c>
-      <c r="F20" s="32" t="n">
+      <c r="G20" s="32" t="n">
         <v>46500000</v>
       </c>
-      <c r="G20" s="33" t="n">
+      <c r="H20" s="33" t="n">
         <v>216279.0697674419</v>
       </c>
-      <c r="H20" s="34" t="n">
+      <c r="I20" s="34" t="n">
         <v>0.9488372093023256</v>
       </c>
-      <c r="I20" s="33" t="n">
+      <c r="J20" s="33" t="n">
         <v>1940.772093023256</v>
       </c>
-      <c r="J20" s="34" t="n">
+      <c r="K20" s="34" t="n">
         <v>-0.07013679161485165</v>
       </c>
-      <c r="K20" s="32" t="n">
+      <c r="L20" s="32" t="n">
         <v>2240292</v>
       </c>
-      <c r="L20" s="35" t="n">
+      <c r="M20" s="35" t="n">
         <v>0.04817832258064516</v>
       </c>
-      <c r="M20" s="35" t="n">
+      <c r="N20" s="35" t="n">
         <v>0.04974305591528602</v>
       </c>
-      <c r="N20" s="35" t="n">
+      <c r="O20" s="35" t="n">
         <v>0.05298602966198496</v>
       </c>
-      <c r="O20" s="35" t="n">
+      <c r="P20" s="35" t="n">
         <v>0.05</v>
       </c>
-      <c r="P20" s="34" t="n">
+      <c r="Q20" s="34" t="n">
         <v>0.1638007066406761</v>
       </c>
-      <c r="Q20" s="36" t="n">
+      <c r="R20" s="36" t="n">
         <v>2.024875332077828</v>
       </c>
     </row>
@@ -1245,36 +1270,41 @@
       </c>
       <c r="B21" s="20" t="n"/>
       <c r="C21" s="20" t="n"/>
-      <c r="D21" s="21" t="n">
+      <c r="D21" s="21" t="inlineStr">
+        <is>
+          <t>3 Houston · 1 Miami</t>
+        </is>
+      </c>
+      <c r="E21" s="21" t="n">
         <v>1232</v>
       </c>
-      <c r="E21" s="22" t="inlineStr"/>
-      <c r="F21" s="23" t="n">
+      <c r="F21" s="22" t="inlineStr"/>
+      <c r="G21" s="23" t="n">
         <v>318500000</v>
       </c>
-      <c r="G21" s="24" t="n">
+      <c r="H21" s="24" t="n">
         <v>258522.7272727273</v>
       </c>
-      <c r="H21" s="25" t="n">
+      <c r="I21" s="25" t="n">
         <v>0.9488636363636364</v>
       </c>
-      <c r="I21" s="24" t="inlineStr"/>
-      <c r="J21" s="25" t="inlineStr"/>
-      <c r="K21" s="23" t="n">
+      <c r="J21" s="24" t="inlineStr"/>
+      <c r="K21" s="25" t="inlineStr"/>
+      <c r="L21" s="23" t="n">
         <v>15371745</v>
       </c>
-      <c r="L21" s="26" t="n">
+      <c r="M21" s="26" t="n">
         <v>0.04826293563579278</v>
       </c>
-      <c r="M21" s="26" t="n">
+      <c r="N21" s="26" t="n">
         <v>0.04959583270489495</v>
       </c>
-      <c r="N21" s="26" t="inlineStr"/>
-      <c r="O21" s="26" t="n">
+      <c r="O21" s="26" t="inlineStr"/>
+      <c r="P21" s="26" t="n">
         <v>0.04934595209550115</v>
       </c>
-      <c r="P21" s="25" t="inlineStr"/>
-      <c r="Q21" s="27" t="inlineStr"/>
+      <c r="Q21" s="25" t="inlineStr"/>
+      <c r="R21" s="27" t="inlineStr"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
@@ -1879,12 +1909,12 @@
   </sheetData>
   <mergeCells count="62">
     <mergeCell ref="A13:W13"/>
-    <mergeCell ref="R16:W16"/>
     <mergeCell ref="E10:G10"/>
     <mergeCell ref="A41:C41"/>
     <mergeCell ref="N28:W28"/>
     <mergeCell ref="M10:O10"/>
     <mergeCell ref="D37:V37"/>
+    <mergeCell ref="S16:W16"/>
     <mergeCell ref="A37:C37"/>
     <mergeCell ref="Q10:S10"/>
     <mergeCell ref="A18:C18"/>

</xml_diff>